<commit_message>
added readme, small fixes
</commit_message>
<xml_diff>
--- a/Codes Manual.xlsx
+++ b/Codes Manual.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\David\MIT Dropbox\David Izrailov\MIT\Academics\Spring\RA\Medicaid\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11B04F80-7199-412A-8F75-55448AE6708C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B4C375-BF04-4E04-8FC9-73FE0D9B4778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{366E5D01-D3F5-1348-8316-7A09D009B710}"/>
+    <workbookView xWindow="-31860" yWindow="5895" windowWidth="28800" windowHeight="15345" xr2:uid="{366E5D01-D3F5-1348-8316-7A09D009B710}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="248">
   <si>
     <t>Cardiovagal (heart rate variability with deep breathing)</t>
   </si>
@@ -803,6 +803,66 @@
   </si>
   <si>
     <t>electrophysiologic evaluation of a subcutaneous implantable cardioverter-defibrillator</t>
+  </si>
+  <si>
+    <t>A0425</t>
+  </si>
+  <si>
+    <t>A0426</t>
+  </si>
+  <si>
+    <t>A0427</t>
+  </si>
+  <si>
+    <t>A0428</t>
+  </si>
+  <si>
+    <t>A0429</t>
+  </si>
+  <si>
+    <t>A0433</t>
+  </si>
+  <si>
+    <t>A0434</t>
+  </si>
+  <si>
+    <t>Advanced Life Support (ALS), non-emergency transport (Level 1)</t>
+  </si>
+  <si>
+    <t>Advanced Life Support (ALS), emergency transport (Level 1)</t>
+  </si>
+  <si>
+    <t>Basic Life Support (BLS), non-emergency transport</t>
+  </si>
+  <si>
+    <t>Basic Life Support (BLS), emergency transport</t>
+  </si>
+  <si>
+    <t>Ground mileage (per statute mile)</t>
+  </si>
+  <si>
+    <t>Advanced Life Support, Level 2 (ALS2) – requires multiple specific interventions</t>
+  </si>
+  <si>
+    <t>Specialty Care Transport (SCT)</t>
+  </si>
+  <si>
+    <t>A0430</t>
+  </si>
+  <si>
+    <t>A0431</t>
+  </si>
+  <si>
+    <t>A0422</t>
+  </si>
+  <si>
+    <t>Conventional air services, transport, one way (fixed wing)</t>
+  </si>
+  <si>
+    <t>Conventional air services, transport, one way (rotary wing / helicopter)</t>
+  </si>
+  <si>
+    <t>Ambulance oxygen and supplies (life-sustaining)</t>
   </si>
 </sst>
 </file>
@@ -4574,6 +4634,116 @@
         <v>168</v>
       </c>
     </row>
+    <row r="295" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A295" t="s">
+        <v>228</v>
+      </c>
+      <c r="B295" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="C295" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="296" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A296" t="s">
+        <v>229</v>
+      </c>
+      <c r="B296" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="C296" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A297" t="s">
+        <v>230</v>
+      </c>
+      <c r="B297" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="C297" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A298" t="s">
+        <v>231</v>
+      </c>
+      <c r="B298" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="C298" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A299" t="s">
+        <v>232</v>
+      </c>
+      <c r="B299" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="C299" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A300" t="s">
+        <v>233</v>
+      </c>
+      <c r="B300" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="C300" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A301" t="s">
+        <v>234</v>
+      </c>
+      <c r="B301" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="C301" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A302" t="s">
+        <v>242</v>
+      </c>
+      <c r="B302" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="C302" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A303" t="s">
+        <v>243</v>
+      </c>
+      <c r="B303" t="s">
+        <v>246</v>
+      </c>
+      <c r="C303" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A304" t="s">
+        <v>244</v>
+      </c>
+      <c r="B304" t="s">
+        <v>247</v>
+      </c>
+      <c r="C304" t="s">
+        <v>168</v>
+      </c>
+    </row>
     <row r="319" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A319" s="1"/>
     </row>
@@ -5517,7 +5687,7 @@
   <conditionalFormatting sqref="A1:A289 A319:A1048576 A292">
     <cfRule type="duplicateValues" dxfId="4" priority="12"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A1048576">
+  <conditionalFormatting sqref="A1:A298 A300:A1048576">
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A289 A319:A631 A292">

</xml_diff>

<commit_message>
updated vline for bars
</commit_message>
<xml_diff>
--- a/Codes Manual.xlsx
+++ b/Codes Manual.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\David\MIT Dropbox\David Izrailov\MIT\Academics\Spring\RA\Medicaid\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B4C375-BF04-4E04-8FC9-73FE0D9B4778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D702E54-18B1-4B86-8C48-118490895564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-31860" yWindow="5895" windowWidth="28800" windowHeight="15345" xr2:uid="{366E5D01-D3F5-1348-8316-7A09D009B710}"/>
+    <workbookView xWindow="9510" yWindow="2070" windowWidth="28800" windowHeight="15345" xr2:uid="{366E5D01-D3F5-1348-8316-7A09D009B710}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="256">
   <si>
     <t>Cardiovagal (heart rate variability with deep breathing)</t>
   </si>
@@ -863,6 +863,30 @@
   </si>
   <si>
     <t>Ambulance oxygen and supplies (life-sustaining)</t>
+  </si>
+  <si>
+    <t>Right heart catheterization</t>
+  </si>
+  <si>
+    <t>Troponin quantitative</t>
+  </si>
+  <si>
+    <t>Troponin qualitative</t>
+  </si>
+  <si>
+    <t>Coronary calcium scoring</t>
+  </si>
+  <si>
+    <t>Coronary angiography procedure that includes catheter placement in coronary arteries and bypass grafts</t>
+  </si>
+  <si>
+    <t>Assay of free kappa and lambda light chains</t>
+  </si>
+  <si>
+    <t>Serum immunofixation electrophoresis (IFE)</t>
+  </si>
+  <si>
+    <t>Serum protein electrophoresis (SPEP) and total protein</t>
   </si>
 </sst>
 </file>
@@ -962,7 +986,47 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1343,7 +1407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B7F554C-5CA4-6C44-A342-D470D08D4CF9}">
-  <dimension ref="A1:H631"/>
+  <dimension ref="A1:H628"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="106" style="5" bestFit="1" customWidth="1"/>
@@ -4536,22 +4600,22 @@
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A286" s="1">
-        <v>93452</v>
-      </c>
-      <c r="B286" t="s">
-        <v>219</v>
+      <c r="A286">
+        <v>33270</v>
+      </c>
+      <c r="B286" s="5" t="s">
+        <v>223</v>
       </c>
       <c r="C286" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A287" s="1">
-        <v>93453</v>
+      <c r="A287">
+        <v>33271</v>
       </c>
       <c r="B287" s="5" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C287" t="s">
         <v>168</v>
@@ -4559,21 +4623,21 @@
     </row>
     <row r="288" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A288" s="1">
-        <v>93456</v>
+        <v>33272</v>
       </c>
       <c r="B288" s="5" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C288" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A289" s="1">
-        <v>93460</v>
+      <c r="A289">
+        <v>93281</v>
       </c>
       <c r="B289" s="5" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C289" t="s">
         <v>168</v>
@@ -4581,54 +4645,54 @@
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A290">
-        <v>33270</v>
-      </c>
-      <c r="B290" s="5" t="s">
-        <v>223</v>
+        <v>93644</v>
+      </c>
+      <c r="B290" t="s">
+        <v>227</v>
       </c>
       <c r="C290" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A291">
-        <v>33271</v>
+      <c r="A291" t="s">
+        <v>228</v>
       </c>
       <c r="B291" s="5" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="C291" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A292" s="1">
-        <v>33272</v>
+      <c r="A292" t="s">
+        <v>229</v>
       </c>
       <c r="B292" s="5" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="C292" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A293">
-        <v>93281</v>
+      <c r="A293" t="s">
+        <v>230</v>
       </c>
       <c r="B293" s="5" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="C293" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="294" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A294">
-        <v>93644</v>
-      </c>
-      <c r="B294" t="s">
-        <v>227</v>
+      <c r="A294" t="s">
+        <v>231</v>
+      </c>
+      <c r="B294" s="5" t="s">
+        <v>237</v>
       </c>
       <c r="C294" t="s">
         <v>168</v>
@@ -4636,10 +4700,10 @@
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B295" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C295" t="s">
         <v>168</v>
@@ -4647,10 +4711,10 @@
     </row>
     <row r="296" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B296" s="5" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C296" t="s">
         <v>168</v>
@@ -4658,10 +4722,10 @@
     </row>
     <row r="297" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B297" s="5" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="C297" t="s">
         <v>168</v>
@@ -4669,10 +4733,10 @@
     </row>
     <row r="298" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="B298" s="5" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="C298" t="s">
         <v>168</v>
@@ -4680,10 +4744,10 @@
     </row>
     <row r="299" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>232</v>
-      </c>
-      <c r="B299" s="5" t="s">
-        <v>238</v>
+        <v>243</v>
+      </c>
+      <c r="B299" t="s">
+        <v>246</v>
       </c>
       <c r="C299" t="s">
         <v>168</v>
@@ -4691,63 +4755,171 @@
     </row>
     <row r="300" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>233</v>
-      </c>
-      <c r="B300" s="5" t="s">
-        <v>240</v>
+        <v>244</v>
+      </c>
+      <c r="B300" t="s">
+        <v>247</v>
       </c>
       <c r="C300" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="301" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A301" t="s">
-        <v>234</v>
+      <c r="A301">
+        <v>93541</v>
       </c>
       <c r="B301" s="5" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="C301" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="302" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A302" t="s">
-        <v>242</v>
-      </c>
-      <c r="B302" s="5" t="s">
-        <v>245</v>
+      <c r="A302" s="1">
+        <v>93452</v>
+      </c>
+      <c r="B302" t="s">
+        <v>219</v>
       </c>
       <c r="C302" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="303" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A303" t="s">
-        <v>243</v>
-      </c>
-      <c r="B303" t="s">
-        <v>246</v>
+      <c r="A303" s="1">
+        <v>93453</v>
+      </c>
+      <c r="B303" s="5" t="s">
+        <v>220</v>
       </c>
       <c r="C303" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="304" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A304" t="s">
-        <v>244</v>
-      </c>
-      <c r="B304" t="s">
-        <v>247</v>
+      <c r="A304" s="1">
+        <v>93456</v>
+      </c>
+      <c r="B304" s="5" t="s">
+        <v>221</v>
       </c>
       <c r="C304" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="319" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A305" s="1">
+        <v>93457</v>
+      </c>
+      <c r="B305" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C305" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A306" s="1">
+        <v>93460</v>
+      </c>
+      <c r="B306" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="C306" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A307">
+        <v>84484</v>
+      </c>
+      <c r="B307" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="C307" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A308">
+        <v>84512</v>
+      </c>
+      <c r="B308" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="C308" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A309">
+        <v>75571</v>
+      </c>
+      <c r="B309" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="C309" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A310">
+        <v>83521</v>
+      </c>
+      <c r="B310" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="C310" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A311">
+        <v>86334</v>
+      </c>
+      <c r="B311" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="C311" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A312">
+        <v>84165</v>
+      </c>
+      <c r="B312" t="s">
+        <v>255</v>
+      </c>
+      <c r="C312" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A313">
+        <v>84155</v>
+      </c>
+      <c r="B313" t="s">
+        <v>255</v>
+      </c>
+      <c r="C313" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A316" s="1"/>
+    </row>
+    <row r="317" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A317" s="1"/>
+    </row>
+    <row r="318" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A318" s="1"/>
+    </row>
+    <row r="319" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A319" s="1"/>
     </row>
-    <row r="320" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A320" s="1"/>
     </row>
     <row r="321" spans="1:1" x14ac:dyDescent="0.25">
@@ -5674,26 +5846,23 @@
     <row r="628" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A628" s="1"/>
     </row>
-    <row r="629" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A629" s="1"/>
-    </row>
-    <row r="630" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A630" s="1"/>
-    </row>
-    <row r="631" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A631" s="1"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:A289 A319:A1048576 A292">
-    <cfRule type="duplicateValues" dxfId="4" priority="12"/>
+  <conditionalFormatting sqref="A1:A294 A296:A1048576">
+    <cfRule type="duplicateValues" dxfId="8" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A298 A300:A1048576">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+  <conditionalFormatting sqref="A302">
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A289 A319:A631 A292">
-    <cfRule type="duplicateValues" dxfId="2" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="15"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="16"/>
+  <conditionalFormatting sqref="A316:A628 A2:A285 A303:A306 A288">
+    <cfRule type="duplicateValues" dxfId="3" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="30"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A316:A1048576 A1:A285 A303:A306 A288">
+    <cfRule type="duplicateValues" dxfId="0" priority="21"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>